<commit_message>
feat: merge new UI design with latest player data (50 batters, 30 bowlers, 267 keepers, 31 teams)
</commit_message>
<xml_diff>
--- a/reports/WicketKeepers_latest.xlsx
+++ b/reports/WicketKeepers_latest.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="WicketKeepers" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WicketKeepers" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$1:$I$304</definedName>
@@ -20,13 +20,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -57,7 +60,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -65,16 +68,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -444,62 +456,62 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Club Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Name of Keeper</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Vs Team</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Balls Faced</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Catches</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Stumps</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Out/Not out</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Match Summary</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Captain Yes\No</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>_match_id</t>
         </is>
@@ -15605,86 +15617,86 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Club Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Name of Keeper</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Vs Team</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Balls Faced</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Catches</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Stumps</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Out/Not out</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>16 Jul 2026</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Vijaya Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>ANVAY DRAVID (RHB) (C)(WK)</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Vultures CC (U-19)</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="3" t="n">
         <v>79</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" s="3" t="n">
         <v>71</v>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -15730,39 +15742,39 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>14 Jul 2026</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Vijaya Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>ANVAY DRAVID (RHB) (C)(WK)</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Swastic Union Cricket Club (1) (U-19)</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="3" t="n">
         <v>93</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="H4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -15886,39 +15898,39 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>12 Jul 2026</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Swastic Union Cricket Club (1) (U-19)</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>SAI AKHILESH B (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Social Cricketers (U-19)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="3" t="n">
         <v>43</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F8" s="3" t="n">
         <v>57</v>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="G8" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="H8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -16198,39 +16210,39 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>10 Jul 2026</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Bangalore Sports Club (U-19)</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>ARNAVV SHARMA (RHB) (C)(WK)</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>Neptune Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E16" s="3" t="n">
         <v>124</v>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="F16" s="3" t="n">
         <v>79</v>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="G16" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H16" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="H16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -16822,39 +16834,39 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>08 Jul 2026</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>Swastic Union Cricket Club (2) (U-19)</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>REHAN MOHAMMED (RHB) (C)(WK)</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>Coles Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="E32" s="2" t="n">
+      <c r="E32" s="3" t="n">
         <v>72</v>
       </c>
-      <c r="F32" s="2" t="n">
+      <c r="F32" s="3" t="n">
         <v>101</v>
       </c>
-      <c r="G32" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H32" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="G32" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
         <is>
           <t>Not out</t>
         </is>
@@ -17446,39 +17458,39 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="A48" s="3" t="inlineStr">
         <is>
           <t>04 Jul 2026</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B48" s="3" t="inlineStr">
         <is>
           <t>Jawahar Sp.Club (1) (U-19)</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="C48" s="3" t="inlineStr">
         <is>
           <t>VARUN PATEL LOKESHA (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="D48" s="3" t="inlineStr">
         <is>
           <t>Jawans Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="E48" s="2" t="n">
+      <c r="E48" s="3" t="n">
         <v>42</v>
       </c>
-      <c r="F48" s="2" t="n">
+      <c r="F48" s="3" t="n">
         <v>41</v>
       </c>
-      <c r="G48" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I48" s="2" t="inlineStr">
+      <c r="G48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -17524,39 +17536,39 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="A50" s="3" t="inlineStr">
         <is>
           <t>03 Jul 2026</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>Young Lions Club (U-19)</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="C50" s="3" t="inlineStr">
         <is>
           <t>CHIRAG HARSHA (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="D50" s="3" t="inlineStr">
         <is>
           <t>Sapphire Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="E50" s="2" t="n">
+      <c r="E50" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="F50" s="2" t="n">
+      <c r="F50" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="G50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I50" s="2" t="inlineStr">
+      <c r="G50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" s="3" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -17680,39 +17692,39 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
+      <c r="A54" s="3" t="inlineStr">
         <is>
           <t>02 Jul 2026</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B54" s="3" t="inlineStr">
         <is>
           <t>Malleswaram Gymkhana (U-19)</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="C54" s="3" t="inlineStr">
         <is>
           <t>S GOUTHAM KRISHNA REDDY (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="D54" s="3" t="inlineStr">
         <is>
           <t>Social Cricketers (U-19)</t>
         </is>
       </c>
-      <c r="E54" s="2" t="n">
+      <c r="E54" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F54" s="2" t="n">
+      <c r="F54" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="G54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I54" s="2" t="inlineStr">
+      <c r="G54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="3" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -17836,39 +17848,39 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr">
+      <c r="A58" s="3" t="inlineStr">
         <is>
           <t>01 Jul 2026</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>Young Lions Club (U-19)</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
+      <c r="C58" s="3" t="inlineStr">
         <is>
           <t>CHIRAG HARSHA (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>Coles Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="E58" s="2" t="n">
+      <c r="E58" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="F58" s="2" t="n">
+      <c r="F58" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="G58" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H58" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I58" s="2" t="inlineStr">
+      <c r="G58" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H58" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I58" s="3" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -18148,39 +18160,39 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+      <c r="A66" s="3" t="inlineStr">
         <is>
           <t>30 Jun 2026</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B66" s="3" t="inlineStr">
         <is>
           <t>Cambridge Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C66" s="3" t="inlineStr">
         <is>
           <t>NITHIN R (LHB) (WK)</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="D66" s="3" t="inlineStr">
         <is>
           <t>Swastic Union Cricket Club (2) (U-19)</t>
         </is>
       </c>
-      <c r="E66" s="2" t="n">
+      <c r="E66" s="3" t="n">
         <v>58</v>
       </c>
-      <c r="F66" s="2" t="n">
+      <c r="F66" s="3" t="n">
         <v>56</v>
       </c>
-      <c r="G66" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H66" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I66" s="2" t="inlineStr">
+      <c r="G66" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H66" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" s="3" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -18772,39 +18784,39 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="inlineStr">
+      <c r="A82" s="3" t="inlineStr">
         <is>
           <t>28 Jun 2026</t>
         </is>
       </c>
-      <c r="B82" s="2" t="inlineStr">
+      <c r="B82" s="3" t="inlineStr">
         <is>
           <t>Whirlwind Cricketers (U-19)</t>
         </is>
       </c>
-      <c r="C82" s="2" t="inlineStr">
+      <c r="C82" s="3" t="inlineStr">
         <is>
           <t>NEIL SANTOSH HONNAGUDI (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D82" s="2" t="inlineStr">
+      <c r="D82" s="3" t="inlineStr">
         <is>
           <t>Friends Union CC (1) (U-19)</t>
         </is>
       </c>
-      <c r="E82" s="2" t="n">
+      <c r="E82" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F82" s="2" t="n">
+      <c r="F82" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="G82" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H82" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I82" s="2" t="inlineStr">
+      <c r="G82" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H82" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I82" s="3" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -18928,39 +18940,39 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="inlineStr">
+      <c r="A86" s="3" t="inlineStr">
         <is>
           <t>27 Jun 2026</t>
         </is>
       </c>
-      <c r="B86" s="2" t="inlineStr">
+      <c r="B86" s="3" t="inlineStr">
         <is>
           <t>Chintamani Sports Association (Chintamani) (U-19)</t>
         </is>
       </c>
-      <c r="C86" s="2" t="inlineStr">
+      <c r="C86" s="3" t="inlineStr">
         <is>
           <t>MANAS A BALAJI (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D86" s="2" t="inlineStr">
+      <c r="D86" s="3" t="inlineStr">
         <is>
           <t>Jolly Cricketers (U-19)</t>
         </is>
       </c>
-      <c r="E86" s="2" t="n">
+      <c r="E86" s="3" t="n">
         <v>58</v>
       </c>
-      <c r="F86" s="2" t="n">
+      <c r="F86" s="3" t="n">
         <v>54</v>
       </c>
-      <c r="G86" s="2" t="n">
+      <c r="G86" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H86" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I86" s="2" t="inlineStr">
+      <c r="H86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" s="3" t="inlineStr">
         <is>
           <t>Not out</t>
         </is>
@@ -19084,39 +19096,39 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="inlineStr">
+      <c r="A90" s="3" t="inlineStr">
         <is>
           <t>26 Jun 2026</t>
         </is>
       </c>
-      <c r="B90" s="2" t="inlineStr">
+      <c r="B90" s="3" t="inlineStr">
         <is>
           <t>Swastic Union Cricket Club (1) (U-19)</t>
         </is>
       </c>
-      <c r="C90" s="2" t="inlineStr">
+      <c r="C90" s="3" t="inlineStr">
         <is>
           <t>SAI AKHILESH B (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D90" s="2" t="inlineStr">
+      <c r="D90" s="3" t="inlineStr">
         <is>
           <t>Jayanagar Cricketers (U-19)</t>
         </is>
       </c>
-      <c r="E90" s="2" t="n">
+      <c r="E90" s="3" t="n">
         <v>86</v>
       </c>
-      <c r="F90" s="2" t="n">
+      <c r="F90" s="3" t="n">
         <v>113</v>
       </c>
-      <c r="G90" s="2" t="n">
+      <c r="G90" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H90" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I90" s="2" t="inlineStr">
+      <c r="H90" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I90" s="3" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -19747,39 +19759,39 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="inlineStr">
+      <c r="A107" s="3" t="inlineStr">
         <is>
           <t>25 Jun 2026</t>
         </is>
       </c>
-      <c r="B107" s="2" t="inlineStr">
+      <c r="B107" s="3" t="inlineStr">
         <is>
           <t>City Cricketers (2) (U-19)</t>
         </is>
       </c>
-      <c r="C107" s="2" t="inlineStr">
+      <c r="C107" s="3" t="inlineStr">
         <is>
           <t>DIGANTH U (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D107" s="2" t="inlineStr">
+      <c r="D107" s="3" t="inlineStr">
         <is>
           <t>Cavaliers Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="E107" s="2" t="n">
+      <c r="E107" s="3" t="n">
         <v>160</v>
       </c>
-      <c r="F107" s="2" t="n">
+      <c r="F107" s="3" t="n">
         <v>141</v>
       </c>
-      <c r="G107" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H107" s="2" t="n">
+      <c r="G107" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H107" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="I107" s="2" t="inlineStr">
+      <c r="I107" s="3" t="inlineStr">
         <is>
           <t>Not out</t>
         </is>
@@ -20476,39 +20488,39 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="2" t="inlineStr">
+      <c r="A126" s="3" t="inlineStr">
         <is>
           <t>24 Jun 2026</t>
         </is>
       </c>
-      <c r="B126" s="2" t="inlineStr">
+      <c r="B126" s="3" t="inlineStr">
         <is>
           <t>Bangalore Sports Club (U-19)</t>
         </is>
       </c>
-      <c r="C126" s="2" t="inlineStr">
+      <c r="C126" s="3" t="inlineStr">
         <is>
           <t>ARNAVV SHARMA (RHB) (C)(WK)</t>
         </is>
       </c>
-      <c r="D126" s="2" t="inlineStr">
+      <c r="D126" s="3" t="inlineStr">
         <is>
           <t>Vijaya Cricket Club (Malur) (U-19)</t>
         </is>
       </c>
-      <c r="E126" s="2" t="n">
+      <c r="E126" s="3" t="n">
         <v>87</v>
       </c>
-      <c r="F126" s="2" t="n">
+      <c r="F126" s="3" t="n">
         <v>61</v>
       </c>
-      <c r="G126" s="2" t="n">
+      <c r="G126" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H126" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I126" s="2" t="inlineStr">
+      <c r="H126" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I126" s="3" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -21334,39 +21346,39 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="2" t="inlineStr">
+      <c r="A148" s="3" t="inlineStr">
         <is>
           <t>23 Jun 2026</t>
         </is>
       </c>
-      <c r="B148" s="2" t="inlineStr">
+      <c r="B148" s="3" t="inlineStr">
         <is>
           <t>Vijaya Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="C148" s="2" t="inlineStr">
+      <c r="C148" s="3" t="inlineStr">
         <is>
           <t>UDGEET S NANDAN (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D148" s="2" t="inlineStr">
+      <c r="D148" s="3" t="inlineStr">
         <is>
           <t>YMCA Cricket Club (3) (U-19)</t>
         </is>
       </c>
-      <c r="E148" s="2" t="n">
+      <c r="E148" s="3" t="n">
         <v>147</v>
       </c>
-      <c r="F148" s="2" t="n">
+      <c r="F148" s="3" t="n">
         <v>98</v>
       </c>
-      <c r="G148" s="2" t="n">
+      <c r="G148" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H148" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I148" s="2" t="inlineStr">
+      <c r="H148" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I148" s="3" t="inlineStr">
         <is>
           <t>Not out</t>
         </is>
@@ -22227,39 +22239,39 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="2" t="inlineStr">
+      <c r="A171" s="3" t="inlineStr">
         <is>
           <t>22 Jun 2026</t>
         </is>
       </c>
-      <c r="B171" s="2" t="inlineStr">
+      <c r="B171" s="3" t="inlineStr">
         <is>
           <t>Wilson Garden Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="C171" s="2" t="inlineStr">
+      <c r="C171" s="3" t="inlineStr">
         <is>
           <t>MANISH BENJAMIN JOHN (LHB) (C)(WK)</t>
         </is>
       </c>
-      <c r="D171" s="2" t="inlineStr">
+      <c r="D171" s="3" t="inlineStr">
         <is>
           <t>Freelancers Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="E171" s="2" t="n">
+      <c r="E171" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="F171" s="2" t="n">
+      <c r="F171" s="3" t="n">
         <v>60</v>
       </c>
-      <c r="G171" s="2" t="n">
+      <c r="G171" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H171" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I171" s="2" t="inlineStr">
+      <c r="H171" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I171" s="3" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -23163,39 +23175,39 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="2" t="inlineStr">
+      <c r="A195" s="3" t="inlineStr">
         <is>
           <t>21 Jun 2026</t>
         </is>
       </c>
-      <c r="B195" s="2" t="inlineStr">
+      <c r="B195" s="3" t="inlineStr">
         <is>
           <t>City Cricketers (2) (U-19)</t>
         </is>
       </c>
-      <c r="C195" s="2" t="inlineStr">
+      <c r="C195" s="3" t="inlineStr">
         <is>
           <t>DIGANTH U (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D195" s="2" t="inlineStr">
+      <c r="D195" s="3" t="inlineStr">
         <is>
           <t>Merchants Cricket Club (1) (U-19)</t>
         </is>
       </c>
-      <c r="E195" s="2" t="n">
+      <c r="E195" s="3" t="n">
         <v>74</v>
       </c>
-      <c r="F195" s="2" t="n">
+      <c r="F195" s="3" t="n">
         <v>61</v>
       </c>
-      <c r="G195" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H195" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I195" s="2" t="inlineStr">
+      <c r="G195" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H195" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I195" s="3" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -23475,39 +23487,39 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="2" t="inlineStr">
+      <c r="A203" s="3" t="inlineStr">
         <is>
           <t>20 Jun 2026</t>
         </is>
       </c>
-      <c r="B203" s="2" t="inlineStr">
+      <c r="B203" s="3" t="inlineStr">
         <is>
           <t>Cavaliers Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="C203" s="2" t="inlineStr">
+      <c r="C203" s="3" t="inlineStr">
         <is>
           <t>NITHIN P GOWDA (RHB) (C)(WK)</t>
         </is>
       </c>
-      <c r="D203" s="2" t="inlineStr">
+      <c r="D203" s="3" t="inlineStr">
         <is>
           <t>Sir Syed Cricketers (U-19)</t>
         </is>
       </c>
-      <c r="E203" s="2" t="n">
+      <c r="E203" s="3" t="n">
         <v>59</v>
       </c>
-      <c r="F203" s="2" t="n">
+      <c r="F203" s="3" t="n">
         <v>79</v>
       </c>
-      <c r="G203" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H203" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I203" s="2" t="inlineStr">
+      <c r="G203" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H203" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I203" s="3" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -24021,39 +24033,39 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="2" t="inlineStr">
+      <c r="A217" s="3" t="inlineStr">
         <is>
           <t>19 Jun 2026</t>
         </is>
       </c>
-      <c r="B217" s="2" t="inlineStr">
+      <c r="B217" s="3" t="inlineStr">
         <is>
           <t>Vijaya Cricket Club (Malur) (U-19)</t>
         </is>
       </c>
-      <c r="C217" s="2" t="inlineStr">
+      <c r="C217" s="3" t="inlineStr">
         <is>
           <t>KUTAM CHARAN RAM (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D217" s="2" t="inlineStr">
+      <c r="D217" s="3" t="inlineStr">
         <is>
           <t>South End Sports Club (U-19)</t>
         </is>
       </c>
-      <c r="E217" s="2" t="n">
+      <c r="E217" s="3" t="n">
         <v>134</v>
       </c>
-      <c r="F217" s="2" t="n">
+      <c r="F217" s="3" t="n">
         <v>123</v>
       </c>
-      <c r="G217" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H217" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I217" s="2" t="inlineStr">
+      <c r="G217" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H217" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I217" s="3" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -24801,39 +24813,39 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="2" t="inlineStr">
+      <c r="A237" s="3" t="inlineStr">
         <is>
           <t>18 Jun 2026</t>
         </is>
       </c>
-      <c r="B237" s="2" t="inlineStr">
+      <c r="B237" s="3" t="inlineStr">
         <is>
           <t>Yankees Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="C237" s="2" t="inlineStr">
+      <c r="C237" s="3" t="inlineStr">
         <is>
           <t>B M CHIRAG (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D237" s="2" t="inlineStr">
+      <c r="D237" s="3" t="inlineStr">
         <is>
           <t>Modern Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="E237" s="2" t="n">
+      <c r="E237" s="3" t="n">
         <v>56</v>
       </c>
-      <c r="F237" s="2" t="n">
+      <c r="F237" s="3" t="n">
         <v>49</v>
       </c>
-      <c r="G237" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H237" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I237" s="2" t="inlineStr">
+      <c r="G237" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H237" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I237" s="3" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -25659,39 +25671,39 @@
       </c>
     </row>
     <row r="259">
-      <c r="A259" s="2" t="inlineStr">
+      <c r="A259" s="3" t="inlineStr">
         <is>
           <t>17 Jun 2026</t>
         </is>
       </c>
-      <c r="B259" s="2" t="inlineStr">
+      <c r="B259" s="3" t="inlineStr">
         <is>
           <t>Palar Sports Club (Kolar) (U-19)</t>
         </is>
       </c>
-      <c r="C259" s="2" t="inlineStr">
+      <c r="C259" s="3" t="inlineStr">
         <is>
           <t>RATHIN SANJAY R (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D259" s="2" t="inlineStr">
+      <c r="D259" s="3" t="inlineStr">
         <is>
           <t>Sapphire Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="E259" s="2" t="n">
+      <c r="E259" s="3" t="n">
         <v>69</v>
       </c>
-      <c r="F259" s="2" t="n">
+      <c r="F259" s="3" t="n">
         <v>68</v>
       </c>
-      <c r="G259" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H259" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I259" s="2" t="inlineStr">
+      <c r="G259" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H259" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I259" s="3" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -26517,39 +26529,39 @@
       </c>
     </row>
     <row r="281">
-      <c r="A281" s="2" t="inlineStr">
+      <c r="A281" s="3" t="inlineStr">
         <is>
           <t>16 Jun 2026</t>
         </is>
       </c>
-      <c r="B281" s="2" t="inlineStr">
+      <c r="B281" s="3" t="inlineStr">
         <is>
           <t>Viveknagar Cricketers (U-19)</t>
         </is>
       </c>
-      <c r="C281" s="2" t="inlineStr">
+      <c r="C281" s="3" t="inlineStr">
         <is>
           <t>PRAJEETH SHETTY K (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D281" s="2" t="inlineStr">
+      <c r="D281" s="3" t="inlineStr">
         <is>
           <t>Chintamani Sports Association (Chintamani) (U-19)</t>
         </is>
       </c>
-      <c r="E281" s="2" t="n">
+      <c r="E281" s="3" t="n">
         <v>56</v>
       </c>
-      <c r="F281" s="2" t="n">
+      <c r="F281" s="3" t="n">
         <v>91</v>
       </c>
-      <c r="G281" s="2" t="n">
+      <c r="G281" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H281" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I281" s="2" t="inlineStr">
+      <c r="H281" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I281" s="3" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -27375,39 +27387,39 @@
       </c>
     </row>
     <row r="303">
-      <c r="A303" s="2" t="inlineStr">
+      <c r="A303" s="3" t="inlineStr">
         <is>
           <t>24 May 2026</t>
         </is>
       </c>
-      <c r="B303" s="2" t="inlineStr">
+      <c r="B303" s="3" t="inlineStr">
         <is>
           <t>Sapphire Cricket Club</t>
         </is>
       </c>
-      <c r="C303" s="2" t="inlineStr">
+      <c r="C303" s="3" t="inlineStr">
         <is>
           <t>Jeevan J V (wk)</t>
         </is>
       </c>
-      <c r="D303" s="2" t="inlineStr">
+      <c r="D303" s="3" t="inlineStr">
         <is>
           <t>Bharath Cricket Club</t>
         </is>
       </c>
-      <c r="E303" s="2" t="n">
+      <c r="E303" s="3" t="n">
         <v>65</v>
       </c>
-      <c r="F303" s="2" t="n">
+      <c r="F303" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="G303" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H303" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I303" s="2" t="inlineStr">
+      <c r="G303" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H303" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I303" s="3" t="inlineStr">
         <is>
           <t>Out</t>
         </is>

</xml_diff>

<commit_message>
chore: update reports, logs, and data files
</commit_message>
<xml_diff>
--- a/reports/WicketKeepers_latest.xlsx
+++ b/reports/WicketKeepers_latest.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WicketKeepers" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="WicketKeepers" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$1:$I$304</definedName>
@@ -20,16 +20,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -60,7 +57,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -68,25 +65,16 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -456,62 +444,62 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Club Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Name of Keeper</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Vs Team</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Balls Faced</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Catches</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Stumps</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Out/Not out</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Match Summary</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Captain Yes\No</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>_match_id</t>
         </is>
@@ -15617,86 +15605,86 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Club Name</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Name of Keeper</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Vs Team</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Balls Faced</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Catches</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Stumps</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Out/Not out</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>16 Jul 2026</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Vijaya Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>ANVAY DRAVID (RHB) (C)(WK)</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Vultures CC (U-19)</t>
         </is>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E2" s="2" t="n">
         <v>79</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="F2" s="2" t="n">
         <v>71</v>
       </c>
-      <c r="G2" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="G2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -15742,39 +15730,39 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>14 Jul 2026</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Vijaya Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>ANVAY DRAVID (RHB) (C)(WK)</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Swastic Union Cricket Club (1) (U-19)</t>
         </is>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E4" s="2" t="n">
         <v>93</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="F4" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="G4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="H4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -15898,39 +15886,39 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>12 Jul 2026</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Swastic Union Cricket Club (1) (U-19)</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>SAI AKHILESH B (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Social Cricketers (U-19)</t>
         </is>
       </c>
-      <c r="E8" s="3" t="n">
+      <c r="E8" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="F8" s="3" t="n">
+      <c r="F8" s="2" t="n">
         <v>57</v>
       </c>
-      <c r="G8" s="3" t="n">
+      <c r="G8" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="H8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -16210,39 +16198,39 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>10 Jul 2026</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Bangalore Sports Club (U-19)</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>ARNAVV SHARMA (RHB) (C)(WK)</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Neptune Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="E16" s="3" t="n">
+      <c r="E16" s="2" t="n">
         <v>124</v>
       </c>
-      <c r="F16" s="3" t="n">
+      <c r="F16" s="2" t="n">
         <v>79</v>
       </c>
-      <c r="G16" s="3" t="n">
+      <c r="G16" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H16" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="H16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -16834,39 +16822,39 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>08 Jul 2026</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Swastic Union Cricket Club (2) (U-19)</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>REHAN MOHAMMED (RHB) (C)(WK)</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Coles Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="E32" s="3" t="n">
+      <c r="E32" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="F32" s="3" t="n">
+      <c r="F32" s="2" t="n">
         <v>101</v>
       </c>
-      <c r="G32" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H32" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" s="3" t="inlineStr">
+      <c r="G32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>Not out</t>
         </is>
@@ -17458,39 +17446,39 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="inlineStr">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>04 Jul 2026</t>
         </is>
       </c>
-      <c r="B48" s="3" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>Jawahar Sp.Club (1) (U-19)</t>
         </is>
       </c>
-      <c r="C48" s="3" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>VARUN PATEL LOKESHA (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D48" s="3" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>Jawans Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="E48" s="3" t="n">
+      <c r="E48" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="F48" s="3" t="n">
+      <c r="F48" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="G48" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I48" s="3" t="inlineStr">
+      <c r="G48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -17536,39 +17524,39 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="3" t="inlineStr">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>03 Jul 2026</t>
         </is>
       </c>
-      <c r="B50" s="3" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>Young Lions Club (U-19)</t>
         </is>
       </c>
-      <c r="C50" s="3" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>CHIRAG HARSHA (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D50" s="3" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>Sapphire Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="E50" s="3" t="n">
+      <c r="E50" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="F50" s="3" t="n">
+      <c r="F50" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="G50" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H50" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I50" s="3" t="inlineStr">
+      <c r="G50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -17692,39 +17680,39 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="3" t="inlineStr">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>02 Jul 2026</t>
         </is>
       </c>
-      <c r="B54" s="3" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>Malleswaram Gymkhana (U-19)</t>
         </is>
       </c>
-      <c r="C54" s="3" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>S GOUTHAM KRISHNA REDDY (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D54" s="3" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>Social Cricketers (U-19)</t>
         </is>
       </c>
-      <c r="E54" s="3" t="n">
+      <c r="E54" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="F54" s="3" t="n">
+      <c r="F54" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="G54" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H54" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I54" s="3" t="inlineStr">
+      <c r="G54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -17848,39 +17836,39 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="inlineStr">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>01 Jul 2026</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>Young Lions Club (U-19)</t>
         </is>
       </c>
-      <c r="C58" s="3" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>CHIRAG HARSHA (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D58" s="3" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>Coles Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="E58" s="3" t="n">
+      <c r="E58" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="F58" s="3" t="n">
+      <c r="F58" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="G58" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H58" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="I58" s="3" t="inlineStr">
+      <c r="G58" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H58" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -18160,39 +18148,39 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="3" t="inlineStr">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>30 Jun 2026</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>Cambridge Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="C66" s="3" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>NITHIN R (LHB) (WK)</t>
         </is>
       </c>
-      <c r="D66" s="3" t="inlineStr">
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>Swastic Union Cricket Club (2) (U-19)</t>
         </is>
       </c>
-      <c r="E66" s="3" t="n">
+      <c r="E66" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="F66" s="3" t="n">
+      <c r="F66" s="2" t="n">
         <v>56</v>
       </c>
-      <c r="G66" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H66" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I66" s="3" t="inlineStr">
+      <c r="G66" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -18784,39 +18772,39 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="3" t="inlineStr">
+      <c r="A82" s="2" t="inlineStr">
         <is>
           <t>28 Jun 2026</t>
         </is>
       </c>
-      <c r="B82" s="3" t="inlineStr">
+      <c r="B82" s="2" t="inlineStr">
         <is>
           <t>Whirlwind Cricketers (U-19)</t>
         </is>
       </c>
-      <c r="C82" s="3" t="inlineStr">
+      <c r="C82" s="2" t="inlineStr">
         <is>
           <t>NEIL SANTOSH HONNAGUDI (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D82" s="3" t="inlineStr">
+      <c r="D82" s="2" t="inlineStr">
         <is>
           <t>Friends Union CC (1) (U-19)</t>
         </is>
       </c>
-      <c r="E82" s="3" t="n">
+      <c r="E82" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="F82" s="3" t="n">
+      <c r="F82" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="G82" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H82" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I82" s="3" t="inlineStr">
+      <c r="G82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -18940,39 +18928,39 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="3" t="inlineStr">
+      <c r="A86" s="2" t="inlineStr">
         <is>
           <t>27 Jun 2026</t>
         </is>
       </c>
-      <c r="B86" s="3" t="inlineStr">
+      <c r="B86" s="2" t="inlineStr">
         <is>
           <t>Chintamani Sports Association (Chintamani) (U-19)</t>
         </is>
       </c>
-      <c r="C86" s="3" t="inlineStr">
+      <c r="C86" s="2" t="inlineStr">
         <is>
           <t>MANAS A BALAJI (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D86" s="3" t="inlineStr">
+      <c r="D86" s="2" t="inlineStr">
         <is>
           <t>Jolly Cricketers (U-19)</t>
         </is>
       </c>
-      <c r="E86" s="3" t="n">
+      <c r="E86" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="F86" s="3" t="n">
+      <c r="F86" s="2" t="n">
         <v>54</v>
       </c>
-      <c r="G86" s="3" t="n">
+      <c r="G86" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H86" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I86" s="3" t="inlineStr">
+      <c r="H86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
         <is>
           <t>Not out</t>
         </is>
@@ -19096,39 +19084,39 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="3" t="inlineStr">
+      <c r="A90" s="2" t="inlineStr">
         <is>
           <t>26 Jun 2026</t>
         </is>
       </c>
-      <c r="B90" s="3" t="inlineStr">
+      <c r="B90" s="2" t="inlineStr">
         <is>
           <t>Swastic Union Cricket Club (1) (U-19)</t>
         </is>
       </c>
-      <c r="C90" s="3" t="inlineStr">
+      <c r="C90" s="2" t="inlineStr">
         <is>
           <t>SAI AKHILESH B (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D90" s="3" t="inlineStr">
+      <c r="D90" s="2" t="inlineStr">
         <is>
           <t>Jayanagar Cricketers (U-19)</t>
         </is>
       </c>
-      <c r="E90" s="3" t="n">
+      <c r="E90" s="2" t="n">
         <v>86</v>
       </c>
-      <c r="F90" s="3" t="n">
+      <c r="F90" s="2" t="n">
         <v>113</v>
       </c>
-      <c r="G90" s="3" t="n">
+      <c r="G90" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H90" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I90" s="3" t="inlineStr">
+      <c r="H90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -19759,39 +19747,39 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="3" t="inlineStr">
+      <c r="A107" s="2" t="inlineStr">
         <is>
           <t>25 Jun 2026</t>
         </is>
       </c>
-      <c r="B107" s="3" t="inlineStr">
+      <c r="B107" s="2" t="inlineStr">
         <is>
           <t>City Cricketers (2) (U-19)</t>
         </is>
       </c>
-      <c r="C107" s="3" t="inlineStr">
+      <c r="C107" s="2" t="inlineStr">
         <is>
           <t>DIGANTH U (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D107" s="3" t="inlineStr">
+      <c r="D107" s="2" t="inlineStr">
         <is>
           <t>Cavaliers Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="E107" s="3" t="n">
+      <c r="E107" s="2" t="n">
         <v>160</v>
       </c>
-      <c r="F107" s="3" t="n">
+      <c r="F107" s="2" t="n">
         <v>141</v>
       </c>
-      <c r="G107" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H107" s="3" t="n">
+      <c r="G107" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H107" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="I107" s="3" t="inlineStr">
+      <c r="I107" s="2" t="inlineStr">
         <is>
           <t>Not out</t>
         </is>
@@ -20488,39 +20476,39 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="3" t="inlineStr">
+      <c r="A126" s="2" t="inlineStr">
         <is>
           <t>24 Jun 2026</t>
         </is>
       </c>
-      <c r="B126" s="3" t="inlineStr">
+      <c r="B126" s="2" t="inlineStr">
         <is>
           <t>Bangalore Sports Club (U-19)</t>
         </is>
       </c>
-      <c r="C126" s="3" t="inlineStr">
+      <c r="C126" s="2" t="inlineStr">
         <is>
           <t>ARNAVV SHARMA (RHB) (C)(WK)</t>
         </is>
       </c>
-      <c r="D126" s="3" t="inlineStr">
+      <c r="D126" s="2" t="inlineStr">
         <is>
           <t>Vijaya Cricket Club (Malur) (U-19)</t>
         </is>
       </c>
-      <c r="E126" s="3" t="n">
+      <c r="E126" s="2" t="n">
         <v>87</v>
       </c>
-      <c r="F126" s="3" t="n">
+      <c r="F126" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="G126" s="3" t="n">
+      <c r="G126" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H126" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I126" s="3" t="inlineStr">
+      <c r="H126" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I126" s="2" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -21346,39 +21334,39 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="3" t="inlineStr">
+      <c r="A148" s="2" t="inlineStr">
         <is>
           <t>23 Jun 2026</t>
         </is>
       </c>
-      <c r="B148" s="3" t="inlineStr">
+      <c r="B148" s="2" t="inlineStr">
         <is>
           <t>Vijaya Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="C148" s="3" t="inlineStr">
+      <c r="C148" s="2" t="inlineStr">
         <is>
           <t>UDGEET S NANDAN (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D148" s="3" t="inlineStr">
+      <c r="D148" s="2" t="inlineStr">
         <is>
           <t>YMCA Cricket Club (3) (U-19)</t>
         </is>
       </c>
-      <c r="E148" s="3" t="n">
+      <c r="E148" s="2" t="n">
         <v>147</v>
       </c>
-      <c r="F148" s="3" t="n">
+      <c r="F148" s="2" t="n">
         <v>98</v>
       </c>
-      <c r="G148" s="3" t="n">
+      <c r="G148" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H148" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="I148" s="3" t="inlineStr">
+      <c r="H148" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I148" s="2" t="inlineStr">
         <is>
           <t>Not out</t>
         </is>
@@ -22239,39 +22227,39 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="3" t="inlineStr">
+      <c r="A171" s="2" t="inlineStr">
         <is>
           <t>22 Jun 2026</t>
         </is>
       </c>
-      <c r="B171" s="3" t="inlineStr">
+      <c r="B171" s="2" t="inlineStr">
         <is>
           <t>Wilson Garden Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="C171" s="3" t="inlineStr">
+      <c r="C171" s="2" t="inlineStr">
         <is>
           <t>MANISH BENJAMIN JOHN (LHB) (C)(WK)</t>
         </is>
       </c>
-      <c r="D171" s="3" t="inlineStr">
+      <c r="D171" s="2" t="inlineStr">
         <is>
           <t>Freelancers Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="E171" s="3" t="n">
+      <c r="E171" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="F171" s="3" t="n">
+      <c r="F171" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="G171" s="3" t="n">
+      <c r="G171" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H171" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I171" s="3" t="inlineStr">
+      <c r="H171" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I171" s="2" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -23175,39 +23163,39 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="3" t="inlineStr">
+      <c r="A195" s="2" t="inlineStr">
         <is>
           <t>21 Jun 2026</t>
         </is>
       </c>
-      <c r="B195" s="3" t="inlineStr">
+      <c r="B195" s="2" t="inlineStr">
         <is>
           <t>City Cricketers (2) (U-19)</t>
         </is>
       </c>
-      <c r="C195" s="3" t="inlineStr">
+      <c r="C195" s="2" t="inlineStr">
         <is>
           <t>DIGANTH U (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D195" s="3" t="inlineStr">
+      <c r="D195" s="2" t="inlineStr">
         <is>
           <t>Merchants Cricket Club (1) (U-19)</t>
         </is>
       </c>
-      <c r="E195" s="3" t="n">
+      <c r="E195" s="2" t="n">
         <v>74</v>
       </c>
-      <c r="F195" s="3" t="n">
+      <c r="F195" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="G195" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H195" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I195" s="3" t="inlineStr">
+      <c r="G195" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H195" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I195" s="2" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -23487,39 +23475,39 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="3" t="inlineStr">
+      <c r="A203" s="2" t="inlineStr">
         <is>
           <t>20 Jun 2026</t>
         </is>
       </c>
-      <c r="B203" s="3" t="inlineStr">
+      <c r="B203" s="2" t="inlineStr">
         <is>
           <t>Cavaliers Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="C203" s="3" t="inlineStr">
+      <c r="C203" s="2" t="inlineStr">
         <is>
           <t>NITHIN P GOWDA (RHB) (C)(WK)</t>
         </is>
       </c>
-      <c r="D203" s="3" t="inlineStr">
+      <c r="D203" s="2" t="inlineStr">
         <is>
           <t>Sir Syed Cricketers (U-19)</t>
         </is>
       </c>
-      <c r="E203" s="3" t="n">
+      <c r="E203" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="F203" s="3" t="n">
+      <c r="F203" s="2" t="n">
         <v>79</v>
       </c>
-      <c r="G203" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H203" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I203" s="3" t="inlineStr">
+      <c r="G203" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H203" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I203" s="2" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -24033,39 +24021,39 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="3" t="inlineStr">
+      <c r="A217" s="2" t="inlineStr">
         <is>
           <t>19 Jun 2026</t>
         </is>
       </c>
-      <c r="B217" s="3" t="inlineStr">
+      <c r="B217" s="2" t="inlineStr">
         <is>
           <t>Vijaya Cricket Club (Malur) (U-19)</t>
         </is>
       </c>
-      <c r="C217" s="3" t="inlineStr">
+      <c r="C217" s="2" t="inlineStr">
         <is>
           <t>KUTAM CHARAN RAM (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D217" s="3" t="inlineStr">
+      <c r="D217" s="2" t="inlineStr">
         <is>
           <t>South End Sports Club (U-19)</t>
         </is>
       </c>
-      <c r="E217" s="3" t="n">
+      <c r="E217" s="2" t="n">
         <v>134</v>
       </c>
-      <c r="F217" s="3" t="n">
+      <c r="F217" s="2" t="n">
         <v>123</v>
       </c>
-      <c r="G217" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H217" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I217" s="3" t="inlineStr">
+      <c r="G217" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H217" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I217" s="2" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -24813,39 +24801,39 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="3" t="inlineStr">
+      <c r="A237" s="2" t="inlineStr">
         <is>
           <t>18 Jun 2026</t>
         </is>
       </c>
-      <c r="B237" s="3" t="inlineStr">
+      <c r="B237" s="2" t="inlineStr">
         <is>
           <t>Yankees Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="C237" s="3" t="inlineStr">
+      <c r="C237" s="2" t="inlineStr">
         <is>
           <t>B M CHIRAG (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D237" s="3" t="inlineStr">
+      <c r="D237" s="2" t="inlineStr">
         <is>
           <t>Modern Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="E237" s="3" t="n">
+      <c r="E237" s="2" t="n">
         <v>56</v>
       </c>
-      <c r="F237" s="3" t="n">
+      <c r="F237" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="G237" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H237" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I237" s="3" t="inlineStr">
+      <c r="G237" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H237" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I237" s="2" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -25671,39 +25659,39 @@
       </c>
     </row>
     <row r="259">
-      <c r="A259" s="3" t="inlineStr">
+      <c r="A259" s="2" t="inlineStr">
         <is>
           <t>17 Jun 2026</t>
         </is>
       </c>
-      <c r="B259" s="3" t="inlineStr">
+      <c r="B259" s="2" t="inlineStr">
         <is>
           <t>Palar Sports Club (Kolar) (U-19)</t>
         </is>
       </c>
-      <c r="C259" s="3" t="inlineStr">
+      <c r="C259" s="2" t="inlineStr">
         <is>
           <t>RATHIN SANJAY R (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D259" s="3" t="inlineStr">
+      <c r="D259" s="2" t="inlineStr">
         <is>
           <t>Sapphire Cricket Club (U-19)</t>
         </is>
       </c>
-      <c r="E259" s="3" t="n">
+      <c r="E259" s="2" t="n">
         <v>69</v>
       </c>
-      <c r="F259" s="3" t="n">
+      <c r="F259" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G259" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H259" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="I259" s="3" t="inlineStr">
+      <c r="G259" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H259" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I259" s="2" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -26529,39 +26517,39 @@
       </c>
     </row>
     <row r="281">
-      <c r="A281" s="3" t="inlineStr">
+      <c r="A281" s="2" t="inlineStr">
         <is>
           <t>16 Jun 2026</t>
         </is>
       </c>
-      <c r="B281" s="3" t="inlineStr">
+      <c r="B281" s="2" t="inlineStr">
         <is>
           <t>Viveknagar Cricketers (U-19)</t>
         </is>
       </c>
-      <c r="C281" s="3" t="inlineStr">
+      <c r="C281" s="2" t="inlineStr">
         <is>
           <t>PRAJEETH SHETTY K (RHB) (WK)</t>
         </is>
       </c>
-      <c r="D281" s="3" t="inlineStr">
+      <c r="D281" s="2" t="inlineStr">
         <is>
           <t>Chintamani Sports Association (Chintamani) (U-19)</t>
         </is>
       </c>
-      <c r="E281" s="3" t="n">
+      <c r="E281" s="2" t="n">
         <v>56</v>
       </c>
-      <c r="F281" s="3" t="n">
+      <c r="F281" s="2" t="n">
         <v>91</v>
       </c>
-      <c r="G281" s="3" t="n">
+      <c r="G281" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H281" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I281" s="3" t="inlineStr">
+      <c r="H281" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I281" s="2" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
@@ -27387,39 +27375,39 @@
       </c>
     </row>
     <row r="303">
-      <c r="A303" s="3" t="inlineStr">
+      <c r="A303" s="2" t="inlineStr">
         <is>
           <t>24 May 2026</t>
         </is>
       </c>
-      <c r="B303" s="3" t="inlineStr">
+      <c r="B303" s="2" t="inlineStr">
         <is>
           <t>Sapphire Cricket Club</t>
         </is>
       </c>
-      <c r="C303" s="3" t="inlineStr">
+      <c r="C303" s="2" t="inlineStr">
         <is>
           <t>Jeevan J V (wk)</t>
         </is>
       </c>
-      <c r="D303" s="3" t="inlineStr">
+      <c r="D303" s="2" t="inlineStr">
         <is>
           <t>Bharath Cricket Club</t>
         </is>
       </c>
-      <c r="E303" s="3" t="n">
+      <c r="E303" s="2" t="n">
         <v>65</v>
       </c>
-      <c r="F303" s="3" t="n">
+      <c r="F303" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="G303" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H303" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="I303" s="3" t="inlineStr">
+      <c r="G303" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H303" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I303" s="2" t="inlineStr">
         <is>
           <t>Out</t>
         </is>

</xml_diff>